<commit_message>
Got a version that pulls up a web browser
</commit_message>
<xml_diff>
--- a/Testing_links_incentivai.xlsx
+++ b/Testing_links_incentivai.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dawso\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dawso\Downloads\Github_work\IncentivAI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9843CED-7EEC-4BD5-8F4B-519D25E5D75D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F73DEBC5-DA00-4E35-B263-00065FDA33B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{695C1AA0-4E41-4E17-8F12-C07DD2378673}"/>
   </bookViews>
@@ -36,39 +36,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
-  <si>
-    <t>URL</t>
-  </si>
-  <si>
-    <t>http://www.ci.brenham.tx.us/utilities/uelectric.php</t>
-  </si>
-  <si>
-    <t>http://www.ci.monmouth.or.us/pview.aspx?id=4776</t>
-  </si>
-  <si>
-    <t>http://www.ci.sebastopol.ca.us</t>
-  </si>
-  <si>
-    <t>http://www.city.cleveland.oh.us/CityofCleveland/Home/Government/CityAgencies/CommunityDevelopment/TaxAbatement</t>
-  </si>
-  <si>
-    <t>http://www.cityofchicago.org/city/en/depts/bldgs/supp_info/chicago-energy-conservation-code.html</t>
-  </si>
-  <si>
-    <t>http://www.cityofchicago.org/city/en/progs/env/solar_in_chicago.html</t>
-  </si>
-  <si>
-    <t>http://www.cityofchicago.org/content/dam/city/depts/zlup/Sustainable_Development/Publications/City_of_Chicago_Solar_Zoning_Policy_Updated.pdf</t>
-  </si>
-  <si>
-    <t>http://www.cityofdubuque.org/index.aspx?NID=1464</t>
-  </si>
-  <si>
-    <t>http://www.cityoflompoc.com/utilities/conservation/</t>
-  </si>
-  <si>
-    <t>http://www.cleanwisconsin.org/index.php?module=cms&amp;page=805</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+  <si>
+    <t>https://www.anaheim.net/3312/Public-EV-Charger-Rebate</t>
+  </si>
+  <si>
+    <t>https://www.aikenco-op.org/water-heater</t>
+  </si>
+  <si>
+    <t>check if it can get open up tabs</t>
+  </si>
+  <si>
+    <t>https://cpi1.gpfulfillment.com/</t>
+  </si>
+  <si>
+    <t>https://beachesenergy.com/my-account/energy-rebates</t>
+  </si>
+  <si>
+    <t>https://www.cedarburglightandwater.org/shared-savings-program</t>
+  </si>
+  <si>
+    <t>URLs</t>
   </si>
 </sst>
 </file>
@@ -447,83 +435,61 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BFA5405-D73C-4729-8263-C7140667B5A8}">
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
-      <c r="A2" s="1" t="s">
+    <row r="3" spans="1:8">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
-      <c r="A3" s="1" t="s">
+    <row r="4" spans="1:8">
+      <c r="A4" s="1"/>
+      <c r="H4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
-      <c r="A4" s="1" t="s">
+    <row r="5" spans="1:8">
+      <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
-      <c r="A5" s="1" t="s">
+    <row r="6" spans="1:8">
+      <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
-      <c r="A6" s="1" t="s">
+    <row r="7" spans="1:8">
+      <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:1">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1">
-      <c r="A8" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1">
-      <c r="A9" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1">
-      <c r="A10" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1">
-      <c r="A11" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1">
-      <c r="A12" s="1" t="s">
-        <v>10</v>
-      </c>
+    <row r="8" spans="1:8">
+      <c r="A8" s="1"/>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="1"/>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="1"/>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="1"/>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="1"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{858DDCEB-E0CD-4830-A1CD-03542AB30ABC}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{15350610-E414-4692-B57C-8D97E0DA655D}"/>
-    <hyperlink ref="A4" r:id="rId3" xr:uid="{43639B11-7F76-4D25-B265-25BE3C277F84}"/>
-    <hyperlink ref="A5" r:id="rId4" xr:uid="{EB5D25E2-4E5F-4829-BF86-E339A2CC0CA8}"/>
-    <hyperlink ref="A6" r:id="rId5" xr:uid="{08070603-B713-44C5-8DA9-7381961EE7AC}"/>
-    <hyperlink ref="A7" r:id="rId6" xr:uid="{B4C18D9E-E5C5-4FB5-A770-24EB64FA293C}"/>
-    <hyperlink ref="A8" r:id="rId7" xr:uid="{ACF50D34-38D1-4498-B3C6-EA14EE622155}"/>
-    <hyperlink ref="A9" r:id="rId8" xr:uid="{A36F11A2-5728-4D66-BFC2-65105E873466}"/>
-    <hyperlink ref="A10" r:id="rId9" xr:uid="{54A1B576-FF99-49B7-A068-009039F5871C}"/>
-    <hyperlink ref="A11" r:id="rId10" xr:uid="{C4767549-BA2D-452E-904D-A84FA542D52F}"/>
-    <hyperlink ref="A12" r:id="rId11" xr:uid="{B3B81284-D920-4949-A771-38D094BEB7C6}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated Coding in my branch. Iteration that has depth but is missing entries
</commit_message>
<xml_diff>
--- a/Testing_links_incentivai.xlsx
+++ b/Testing_links_incentivai.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dawso\Downloads\Github_work\IncentivAI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F73DEBC5-DA00-4E35-B263-00065FDA33B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{816A63F4-271B-48E7-8C3F-C2D7E0CBDC42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{695C1AA0-4E41-4E17-8F12-C07DD2378673}"/>
+    <workbookView xWindow="-27045" yWindow="1905" windowWidth="21600" windowHeight="11430" xr2:uid="{695C1AA0-4E41-4E17-8F12-C07DD2378673}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,27 +36,300 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
-  <si>
-    <t>https://www.anaheim.net/3312/Public-EV-Charger-Rebate</t>
-  </si>
-  <si>
-    <t>https://www.aikenco-op.org/water-heater</t>
-  </si>
-  <si>
-    <t>check if it can get open up tabs</t>
-  </si>
-  <si>
-    <t>https://cpi1.gpfulfillment.com/</t>
-  </si>
-  <si>
-    <t>https://beachesenergy.com/my-account/energy-rebates</t>
-  </si>
-  <si>
-    <t>https://www.cedarburglightandwater.org/shared-savings-program</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="98">
   <si>
     <t>URLs</t>
+  </si>
+  <si>
+    <t>http://anaheim.net/936/Energy-Rebates-Incentives</t>
+  </si>
+  <si>
+    <t>http://apps.sos.wv.gov/adlaw/csr/ruleview.aspx?document=8584</t>
+  </si>
+  <si>
+    <t>http://aspencore.org/grants/</t>
+  </si>
+  <si>
+    <t>http://bcapcodes.org/code-status/state/mississippi/</t>
+  </si>
+  <si>
+    <t>http://bcap-ocean.org/state-country/colorado</t>
+  </si>
+  <si>
+    <t>http://bit.ly/1suoNdB</t>
+  </si>
+  <si>
+    <t>http://bpu.org/rebates/</t>
+  </si>
+  <si>
+    <t>http://buildsagreen.org/</t>
+  </si>
+  <si>
+    <t>http://caec.coop/member-benefits-services/heat-pumps/</t>
+  </si>
+  <si>
+    <t>http://cca.hawaii.gov/pvl/boards/contractor/</t>
+  </si>
+  <si>
+    <t>http://city.milwaukee.gov/MilwaukeeShines#.VRw1e-G86W4</t>
+  </si>
+  <si>
+    <t>http://cleanairfleets.org/programs/alt-fuels-colorado</t>
+  </si>
+  <si>
+    <t>http://cleanairfleets.org/programs/charge-ahead-colorado</t>
+  </si>
+  <si>
+    <t>http://commerceri.com/finance-business/renewable-energy-fund/commercial-scale-projects/</t>
+  </si>
+  <si>
+    <t>http://comptroller.marylandtaxes.com/Public_Services/Agency_Information/Office_of_the_Comptroller/Comptroller_Initiatives/Shop_Maryland_Tax-free_Week/</t>
+  </si>
+  <si>
+    <t>http://copace.com/</t>
+  </si>
+  <si>
+    <t>http://cpuc.ca.gov/energyefficiency/</t>
+  </si>
+  <si>
+    <t>http://crpud.net/ways-to-save/at-work</t>
+  </si>
+  <si>
+    <t>http://dallascityhall.com/departments/sustainabledevelopment/buildinginspection/pages/know_code.aspx</t>
+  </si>
+  <si>
+    <t>http://dced.pa.gov/programs/solar-energy-program-sep/#.WDSKnLIrJhE</t>
+  </si>
+  <si>
+    <t>http://depsc.delaware.gov/delrps.shtml</t>
+  </si>
+  <si>
+    <t>http://depsc.delaware.gov/electric.shtml</t>
+  </si>
+  <si>
+    <t>http://deq.mt.gov/Energy/PropertyTaxIncentives.mcpx</t>
+  </si>
+  <si>
+    <t>http://development.ohio.gov/bs/bs_renewenergy.htm</t>
+  </si>
+  <si>
+    <t>http://dor.mo.gov/business/sales/taxholiday/green/</t>
+  </si>
+  <si>
+    <t>http://dor.wa.gov/content/findtaxesandrates/bandotax</t>
+  </si>
+  <si>
+    <t>http://dor.wa.gov/Content/FindTaxesAndRates/TaxIncentives/IncentivePrograms.aspx#Energy</t>
+  </si>
+  <si>
+    <t>http://energy.gov/lpo/loan-programs-office</t>
+  </si>
+  <si>
+    <t>http://energy.hawaii.gov/energy-efficiency-in-soh</t>
+  </si>
+  <si>
+    <t>http://energy.hawaii.gov/renewable-energy</t>
+  </si>
+  <si>
+    <t>http://energy.maryland.gov/business/Pages/incentives/empowermdcigp.aspx</t>
+  </si>
+  <si>
+    <t>http://energy.maryland.gov/business/Pages/incentives/PVEVprogram.aspx</t>
+  </si>
+  <si>
+    <t>http://energy.maryland.gov/Govt/pages/janeelawton.aspx</t>
+  </si>
+  <si>
+    <t>http://energy.maryland.gov/govt/Pages/smartenergycommunities.aspx</t>
+  </si>
+  <si>
+    <t>http://energy.mo.gov/energy</t>
+  </si>
+  <si>
+    <t>http://energy.nv.gov/Programs/Renewable_Energy_Tax_Abatements/</t>
+  </si>
+  <si>
+    <t>http://energytrust.org/commercial</t>
+  </si>
+  <si>
+    <t>http://energytrust.org/newbuildings</t>
+  </si>
+  <si>
+    <t>http://fortworthtexas.gov/sustainability/</t>
+  </si>
+  <si>
+    <t>http://green.dc.gov/service/buy-green-power</t>
+  </si>
+  <si>
+    <t>http://greenbank.ny.gov/</t>
+  </si>
+  <si>
+    <t>http://greendallas.net/green-buildings/</t>
+  </si>
+  <si>
+    <t>http://greenhoustontx.gov/green-power-program.html</t>
+  </si>
+  <si>
+    <t>http://hdoa.hawaii.gov/agl/alternative-energy-loan-program/</t>
+  </si>
+  <si>
+    <t>http://homeenergysavings.delmarva.com/home-performance-with-energy-star-program</t>
+  </si>
+  <si>
+    <t>http://homeenergysavings.pepco.com/home-performance-with-energy-star-program</t>
+  </si>
+  <si>
+    <t>http://kcc.ks.gov/electric/renewable-energy-standard</t>
+  </si>
+  <si>
+    <t>http://licenseinfo.oregon.gov/</t>
+  </si>
+  <si>
+    <t>http://lodielectric.com/906/Commercial-Rebates</t>
+  </si>
+  <si>
+    <t>http://lodielectric.com/908/Commercial-Programs</t>
+  </si>
+  <si>
+    <t>http://lodielectric.com/909/Residential-Rebates</t>
+  </si>
+  <si>
+    <t>http://longbeach.gov/sustainability/media-library/documents/urban-living/builidings-and-neighborhoods/greenbuildingpolicy/</t>
+  </si>
+  <si>
+    <t>http://ma-eeac.org/</t>
+  </si>
+  <si>
+    <t>http://marbleheadelectric.com/rebates-incentives.html</t>
+  </si>
+  <si>
+    <t>http://masmartsolar.com/</t>
+  </si>
+  <si>
+    <t>http://mgaleg.maryland.gov/mgawebsite/Legislation/Details/hb1255/?ys=2019rs</t>
+  </si>
+  <si>
+    <t>http://mmpa.org/conservation/we-save-business/</t>
+  </si>
+  <si>
+    <t>http://mmpa.org/conservation/we-save-home/</t>
+  </si>
+  <si>
+    <t>http://ny-sun.ny.gov/</t>
+  </si>
+  <si>
+    <t>http://ompa.com/programs/deep/</t>
+  </si>
+  <si>
+    <t>http://palaugov.org/</t>
+  </si>
+  <si>
+    <t>http://pge.com/en/save-energy-and-money/energy-saving-programs/energy-efficiency-programs-for-businesses/energy-efficiency-financing.html</t>
+  </si>
+  <si>
+    <t>http://psc.state.wy.us/</t>
+  </si>
+  <si>
+    <t>http://psc.wi.gov/renewables/WindSitingRules.htm</t>
+  </si>
+  <si>
+    <t>http://publicservice.vermont.gov/electric/interconnection</t>
+  </si>
+  <si>
+    <t>http://publicservice.vermont.gov/renewable_energy/cedf</t>
+  </si>
+  <si>
+    <t>http://publicservice.vermont.gov/renewable_energy/net_metering</t>
+  </si>
+  <si>
+    <t>http://publicservice.vermont.gov/renewable_energy/resources</t>
+  </si>
+  <si>
+    <t>http://puc.nv.gov/Renewable_Energy/Net_Metering/</t>
+  </si>
+  <si>
+    <t>http://puc.nv.gov/Renewable_Energy/Portfolio_Standard/</t>
+  </si>
+  <si>
+    <t>http://rmeb.org/pace.htm</t>
+  </si>
+  <si>
+    <t>http://santaclaraca.gov/index.aspx?page=1046</t>
+  </si>
+  <si>
+    <t>http://secpa.com/rebates</t>
+  </si>
+  <si>
+    <t>http://takechargeva.com/business/default.aspx</t>
+  </si>
+  <si>
+    <t>http://tax.hawaii.gov/geninfo/renewable/</t>
+  </si>
+  <si>
+    <t>http://tax.vermont.gov/business-and-corp/corp-and-business-income-taxes/tax-credits</t>
+  </si>
+  <si>
+    <t>http://tax.vermont.gov/municipal-officials/solar-valuation/everything-you-need-to-know-about-solar</t>
+  </si>
+  <si>
+    <t>http://unitil.com/energy-efficiency/energy-efficiency-programs/natural-gas-programs-rebates-assistance</t>
+  </si>
+  <si>
+    <t>http://wa-portangeles.civicplus.com/790/Residential-Conservation-Rebates</t>
+  </si>
+  <si>
+    <t>http://wellesleyma.gov/799/Energy-Efficiency-Rebates</t>
+  </si>
+  <si>
+    <t>http://wmgld.com/energy-programs/</t>
+  </si>
+  <si>
+    <t>http://www.aacounty.org/Finance/Forms.cfm</t>
+  </si>
+  <si>
+    <t>http://www.ahfc.us/buy/add-options/energy-efficiency-rate-reduction/</t>
+  </si>
+  <si>
+    <t>http://www.ahfc.us/efficiency/energy-programs/weatherization/</t>
+  </si>
+  <si>
+    <t>http://www.ahfc.us/pros/loans/association-loan-program/</t>
+  </si>
+  <si>
+    <t>http://www.aikenco-op.org/water-heater/</t>
+  </si>
+  <si>
+    <t>http://www.alputilities.com/residential/rebates.php</t>
+  </si>
+  <si>
+    <t>http://www.anaheim.net/3312/Public-EV-Charger-Rebate</t>
+  </si>
+  <si>
+    <t>http://www.anaheim.net/5353/Business-Energy-Rebates</t>
+  </si>
+  <si>
+    <t>http://www.anaheim.net/593/Personal-EV-Charger-Rebate</t>
+  </si>
+  <si>
+    <t>http://www.anaheim.net/911/New-Construction-Incentives</t>
+  </si>
+  <si>
+    <t>http://www.anaheim.net/965/Small-Business-Energy-Water-Direct-Insta</t>
+  </si>
+  <si>
+    <t>http://www.arkansas.gov/psc/index.htm</t>
+  </si>
+  <si>
+    <t>http://www.ashland.or.us/Files/SolarBrochure_WebFormat.pdf</t>
+  </si>
+  <si>
+    <t>http://www.austintexas.gov/department/austin-climate-protection-program</t>
+  </si>
+  <si>
+    <t>http://www.azcc.gov/divisions/utilities/electric.asp</t>
+  </si>
+  <si>
+    <t>http://www.bcremc.com/incentives/</t>
   </si>
 </sst>
 </file>
@@ -435,59 +708,518 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BFA5405-D73C-4729-8263-C7140667B5A8}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:A102"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:1">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="1"/>
-      <c r="H4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="1"/>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" s="1"/>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="1"/>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" s="1"/>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="1"/>
+    <row r="8" spans="1:1">
+      <c r="A8" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1">
+      <c r="A32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1">
+      <c r="A34" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1">
+      <c r="A35" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1">
+      <c r="A36" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1">
+      <c r="A38" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1">
+      <c r="A39" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1">
+      <c r="A40" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1">
+      <c r="A41" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1">
+      <c r="A43" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1">
+      <c r="A44" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1">
+      <c r="A45" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1">
+      <c r="A46" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1">
+      <c r="A47" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1">
+      <c r="A48" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1">
+      <c r="A49" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1">
+      <c r="A52" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1">
+      <c r="A53" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1">
+      <c r="A57" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1">
+      <c r="A58" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1">
+      <c r="A59" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1">
+      <c r="A60" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1">
+      <c r="A61" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1">
+      <c r="A62" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1">
+      <c r="A63" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1">
+      <c r="A64" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1">
+      <c r="A65" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1">
+      <c r="A66" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1">
+      <c r="A67" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1">
+      <c r="A68" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1">
+      <c r="A69" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1">
+      <c r="A71" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1">
+      <c r="A73" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1">
+      <c r="A74" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1">
+      <c r="A76" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1">
+      <c r="A77" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1">
+      <c r="A78" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1">
+      <c r="A79" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1">
+      <c r="A80" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1">
+      <c r="A82" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1">
+      <c r="A83" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1">
+      <c r="A84" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1">
+      <c r="A85" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1">
+      <c r="A86" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1">
+      <c r="A87" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1">
+      <c r="A88" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1">
+      <c r="A89" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1">
+      <c r="A90" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1">
+      <c r="A91" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1">
+      <c r="A92" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1">
+      <c r="A93" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1">
+      <c r="A94" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1">
+      <c r="A95" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1">
+      <c r="A96" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1">
+      <c r="A97" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1">
+      <c r="A98" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1">
+      <c r="A99" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1">
+      <c r="A100" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1">
+      <c r="A101" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1">
+      <c r="A102" t="s">
+        <v>97</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>